<commit_message>
feat: improve booking system, navigation fixes, and documentation updates
- Fix booking flow state handling across date, group, confirm, success, and summary steps
- Standardise localStorage booking storage (pulse-bookings) and improve draft handling
- Add dynamic account booking history rendering from localStorage
- Remove static placeholder booking data in account page
- Improve loading state handling for account orders list

- Fix broken navigation between About and Home pages
- Add contact form to About page and introduce contact section
- Improve semantic structure by ensuring proper use of <h1> across pages

- Fix and update site.webmanifest configuration

- Add pseudocode documentation for key logic flows
- Add draw.io flowcharts for booking system architecture and user flow
</commit_message>
<xml_diff>
--- a/assets/data/assets.xlsx
+++ b/assets/data/assets.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mancoll-my.sharepoint.com/personal/1559003_stu_tmc_ac_uk/Documents/Level 3 - Year 1/TERM 3/Unit 15 Website Development/Assignment 2/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_32E5ACE234863C62C4C9FB08A11D07CE090B100A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F7D76D2-3472-4728-B0B9-8F203EE3FA3F}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="11_32E5ACE234863C62C4C9FB08A11D07CE090B100A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32322CD8-D5AC-406C-9C06-5DFB4CE826B2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Asset Table" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -324,7 +323,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="282">
   <si>
     <t>Asset ID</t>
   </si>
@@ -1170,25 +1169,13 @@
   </si>
   <si>
     <t>A027-moonlight-marsh.jpg</t>
-  </si>
-  <si>
-    <t>Total Assets</t>
-  </si>
-  <si>
-    <t>Average File Size (MB)</t>
-  </si>
-  <si>
-    <t>Asset Type Distribution</t>
-  </si>
-  <si>
-    <t>Photo: 16, Illustration: 11</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1200,6 +1187,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1219,10 +1214,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1231,8 +1227,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1246,6 +1246,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1661,7 +1665,7 @@
       <c r="D2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="F2" s="3" t="str">
@@ -1725,7 +1729,7 @@
       <c r="D3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>38</v>
       </c>
       <c r="F3" s="3" t="str">
@@ -1789,7 +1793,7 @@
       <c r="D4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>49</v>
       </c>
       <c r="F4" s="3" t="str">
@@ -1853,7 +1857,7 @@
       <c r="D5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>59</v>
       </c>
       <c r="F5" s="3" t="str">
@@ -1917,7 +1921,7 @@
       <c r="D6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F6" s="3" t="str">
@@ -1981,7 +1985,7 @@
       <c r="D7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>79</v>
       </c>
       <c r="F7" s="3" t="str">
@@ -2045,7 +2049,7 @@
       <c r="D8" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>88</v>
       </c>
       <c r="F8" s="3" t="str">
@@ -2109,7 +2113,7 @@
       <c r="D9" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>99</v>
       </c>
       <c r="F9" s="3" t="str">
@@ -2173,7 +2177,7 @@
       <c r="D10" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>109</v>
       </c>
       <c r="F10" s="3" t="str">
@@ -2237,7 +2241,7 @@
       <c r="D11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>119</v>
       </c>
       <c r="F11" s="3" t="str">
@@ -2301,7 +2305,7 @@
       <c r="D12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>128</v>
       </c>
       <c r="F12" s="3" t="str">
@@ -2365,7 +2369,7 @@
       <c r="D13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>139</v>
       </c>
       <c r="F13" s="3" t="str">
@@ -2429,7 +2433,7 @@
       <c r="D14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>148</v>
       </c>
       <c r="F14" s="3" t="str">
@@ -2493,7 +2497,7 @@
       <c r="D15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>156</v>
       </c>
       <c r="F15" s="3" t="str">
@@ -2557,7 +2561,7 @@
       <c r="D16" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>166</v>
       </c>
       <c r="F16" s="3" t="str">
@@ -2621,7 +2625,7 @@
       <c r="D17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>175</v>
       </c>
       <c r="F17" s="3" t="str">
@@ -2685,7 +2689,7 @@
       <c r="D18" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>185</v>
       </c>
       <c r="F18" s="3" t="str">
@@ -2749,7 +2753,7 @@
       <c r="D19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="4" t="s">
         <v>193</v>
       </c>
       <c r="F19" s="3" t="str">
@@ -2813,7 +2817,7 @@
       <c r="D20" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>202</v>
       </c>
       <c r="F20" s="3" t="str">
@@ -2877,7 +2881,7 @@
       <c r="D21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>211</v>
       </c>
       <c r="F21" s="3" t="str">
@@ -2941,7 +2945,7 @@
       <c r="D22" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="4" t="s">
         <v>220</v>
       </c>
       <c r="F22" s="3" t="str">
@@ -3005,7 +3009,7 @@
       <c r="D23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>229</v>
       </c>
       <c r="F23" s="3" t="str">
@@ -3069,7 +3073,7 @@
       <c r="D24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>239</v>
       </c>
       <c r="F24" s="3" t="str">
@@ -3133,7 +3137,7 @@
       <c r="D25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="4" t="s">
         <v>248</v>
       </c>
       <c r="F25" s="3" t="str">
@@ -3197,7 +3201,7 @@
       <c r="D26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="4" t="s">
         <v>257</v>
       </c>
       <c r="F26" s="3" t="str">
@@ -3261,7 +3265,7 @@
       <c r="D27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="4" t="s">
         <v>266</v>
       </c>
       <c r="F27" s="3" t="str">
@@ -3325,7 +3329,7 @@
       <c r="D28" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="4" t="s">
         <v>275</v>
       </c>
       <c r="F28" s="3" t="str">
@@ -3377,48 +3381,39 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{6A1B6CCB-D7E8-4292-9733-567934F2C3A1}"/>
+    <hyperlink ref="E4" r:id="rId2" xr:uid="{2C4BF967-F370-4FCC-A81E-AA0FB00903D5}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{4F546358-76AB-40E8-A4F0-08A47C569D10}"/>
+    <hyperlink ref="E6" r:id="rId4" xr:uid="{609942AD-9BE8-485B-8EA3-8A4A3205E6D4}"/>
+    <hyperlink ref="E2" r:id="rId5" xr:uid="{F191CC65-19C4-410D-A502-BCC68FCAD369}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{D7A5D10E-3AB1-4F84-9FE5-56713549647D}"/>
+    <hyperlink ref="E8" r:id="rId7" xr:uid="{F0EDDB6B-14E8-477A-8853-F8DEC5422643}"/>
+    <hyperlink ref="E9" r:id="rId8" xr:uid="{D7752A63-9830-447B-AA96-EA452C151F41}"/>
+    <hyperlink ref="E10" r:id="rId9" xr:uid="{59ED404A-037B-4064-AA44-8435F94869FD}"/>
+    <hyperlink ref="E11" r:id="rId10" xr:uid="{C9FEFBD9-7599-4FC0-82E1-7BDB94CF314E}"/>
+    <hyperlink ref="E12" r:id="rId11" xr:uid="{256E0C02-9D82-42BF-85F8-D9AFDBE8EB78}"/>
+    <hyperlink ref="E13" r:id="rId12" xr:uid="{DE21C9E1-4FE3-48CB-91B7-09125DC1963D}"/>
+    <hyperlink ref="E14" r:id="rId13" xr:uid="{C02033C1-2AFF-4C9F-AB81-D7F0D0B8A942}"/>
+    <hyperlink ref="E15" r:id="rId14" xr:uid="{1ED1E2C7-404E-4A14-9E32-49655492AF93}"/>
+    <hyperlink ref="E16" r:id="rId15" xr:uid="{C3416551-F57A-410F-A53A-01C38E7CAB94}"/>
+    <hyperlink ref="E17" r:id="rId16" xr:uid="{54D35800-D732-4635-83BB-83904EBEF9E1}"/>
+    <hyperlink ref="E18" r:id="rId17" xr:uid="{C8689C5D-0B19-4B10-9AEF-4ECD472792B9}"/>
+    <hyperlink ref="E19" r:id="rId18" xr:uid="{1EB28DE0-D1E5-4333-A98F-E18F88109BAB}"/>
+    <hyperlink ref="E20" r:id="rId19" xr:uid="{AED8FF74-42F7-484E-8123-29FE0CA251B7}"/>
+    <hyperlink ref="E21" r:id="rId20" xr:uid="{892DC094-9089-408D-97EA-2EFC9721DF53}"/>
+    <hyperlink ref="E22" r:id="rId21" xr:uid="{C0BC3501-83D1-48B4-8C4A-1D8689A99B90}"/>
+    <hyperlink ref="E23" r:id="rId22" xr:uid="{BF81A061-B10B-4E37-99F2-DE684CC13FA3}"/>
+    <hyperlink ref="E24" r:id="rId23" xr:uid="{E2FCB57D-212F-442C-8305-B7535624AD2C}"/>
+    <hyperlink ref="E25" r:id="rId24" xr:uid="{20023D28-0A0F-4EB3-A2D9-B796E6A4853D}"/>
+    <hyperlink ref="E26" r:id="rId25" xr:uid="{444B17DE-336E-458B-910A-F013A8E77738}"/>
+    <hyperlink ref="E27" r:id="rId26" xr:uid="{363B6210-3D6B-4F6F-ABDD-961D72D6AB85}"/>
+    <hyperlink ref="E28" r:id="rId27" xr:uid="{C018931C-43B6-4D68-BDFF-363B46D54A77}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId28"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId29"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>282</v>
-      </c>
-      <c r="B1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>283</v>
-      </c>
-      <c r="B2">
-        <v>4.58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B3" t="s">
-        <v>285</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>